<commit_message>
Refuerza informe Quarto y script del Taller 2 con validaciones oficiales DANE, orden cronológico y actualiza README maestro
</commit_message>
<xml_diff>
--- a/outputs/2_1_tasas_hombres.xlsx
+++ b/outputs/2_1_tasas_hombres.xlsx
@@ -17,22 +17,22 @@
     <t xml:space="preserve">Tasas (%) y poblaciones</t>
   </si>
   <si>
+    <t xml:space="preserve">Enero - marzo 2023</t>
+  </si>
+  <si>
     <t xml:space="preserve">Abril - junio 2023</t>
   </si>
   <si>
-    <t xml:space="preserve">Enero - marzo 2023</t>
-  </si>
-  <si>
     <t xml:space="preserve">Julio - septiembre 2023</t>
   </si>
   <si>
     <t xml:space="preserve">Octubre - diciembre 2023</t>
   </si>
   <si>
+    <t xml:space="preserve">Enero - marzo 2024</t>
+  </si>
+  <si>
     <t xml:space="preserve">Abril - junio 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enero - marzo 2024</t>
   </si>
   <si>
     <t xml:space="preserve">Julio - septiembre 2024</t>
@@ -425,10 +425,10 @@
         <v>9</v>
       </c>
       <c r="B2" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="C2" t="n">
         <v>76.74</v>
-      </c>
-      <c r="C2" t="n">
-        <v>76.5</v>
       </c>
       <c r="D2" t="n">
         <v>76.84</v>
@@ -437,10 +437,10 @@
         <v>76.49</v>
       </c>
       <c r="F2" t="n">
+        <v>76.27</v>
+      </c>
+      <c r="G2" t="n">
         <v>76.56</v>
-      </c>
-      <c r="G2" t="n">
-        <v>76.27</v>
       </c>
       <c r="H2" t="n">
         <v>76.37</v>
@@ -454,10 +454,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
+        <v>69.48</v>
+      </c>
+      <c r="C3" t="n">
         <v>70.5</v>
-      </c>
-      <c r="C3" t="n">
-        <v>69.48</v>
       </c>
       <c r="D3" t="n">
         <v>70.96</v>
@@ -466,10 +466,10 @@
         <v>70.53</v>
       </c>
       <c r="F3" t="n">
+        <v>68.97</v>
+      </c>
+      <c r="G3" t="n">
         <v>69.88</v>
-      </c>
-      <c r="G3" t="n">
-        <v>68.97</v>
       </c>
       <c r="H3" t="n">
         <v>70.51</v>
@@ -483,10 +483,10 @@
         <v>11</v>
       </c>
       <c r="B4" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="C4" t="n">
         <v>8.14</v>
-      </c>
-      <c r="C4" t="n">
-        <v>9.18</v>
       </c>
       <c r="D4" t="n">
         <v>7.66</v>
@@ -495,10 +495,10 @@
         <v>7.78</v>
       </c>
       <c r="F4" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="G4" t="n">
         <v>8.72</v>
-      </c>
-      <c r="G4" t="n">
-        <v>9.57</v>
       </c>
       <c r="H4" t="n">
         <v>7.67</v>
@@ -512,10 +512,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="n">
+        <v>24748804</v>
+      </c>
+      <c r="C5" t="n">
         <v>24810197</v>
-      </c>
-      <c r="C5" t="n">
-        <v>24748804</v>
       </c>
       <c r="D5" t="n">
         <v>24869525</v>
@@ -524,10 +524,10 @@
         <v>24930631</v>
       </c>
       <c r="F5" t="n">
+        <v>24990309</v>
+      </c>
+      <c r="G5" t="n">
         <v>25049813</v>
-      </c>
-      <c r="G5" t="n">
-        <v>24990309</v>
       </c>
       <c r="H5" t="n">
         <v>25107634</v>
@@ -541,10 +541,10 @@
         <v>13</v>
       </c>
       <c r="B6" t="n">
+        <v>18881919</v>
+      </c>
+      <c r="C6" t="n">
         <v>18946514</v>
-      </c>
-      <c r="C6" t="n">
-        <v>18881919</v>
       </c>
       <c r="D6" t="n">
         <v>19011565</v>
@@ -553,10 +553,10 @@
         <v>19080726</v>
       </c>
       <c r="F6" t="n">
+        <v>19149619</v>
+      </c>
+      <c r="G6" t="n">
         <v>19218233</v>
-      </c>
-      <c r="G6" t="n">
-        <v>19149619</v>
       </c>
       <c r="H6" t="n">
         <v>19283702</v>
@@ -570,10 +570,10 @@
         <v>14</v>
       </c>
       <c r="B7" t="n">
+        <v>14444388</v>
+      </c>
+      <c r="C7" t="n">
         <v>14540454</v>
-      </c>
-      <c r="C7" t="n">
-        <v>14444388</v>
       </c>
       <c r="D7" t="n">
         <v>14609435</v>
@@ -582,10 +582,10 @@
         <v>14594473</v>
       </c>
       <c r="F7" t="n">
+        <v>14604582</v>
+      </c>
+      <c r="G7" t="n">
         <v>14712896</v>
-      </c>
-      <c r="G7" t="n">
-        <v>14604582</v>
       </c>
       <c r="H7" t="n">
         <v>14726116</v>
@@ -599,10 +599,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="n">
+        <v>13118794</v>
+      </c>
+      <c r="C8" t="n">
         <v>13357249</v>
-      </c>
-      <c r="C8" t="n">
-        <v>13118794</v>
       </c>
       <c r="D8" t="n">
         <v>13490093</v>
@@ -611,10 +611,10 @@
         <v>13458585</v>
       </c>
       <c r="F8" t="n">
+        <v>13207089</v>
+      </c>
+      <c r="G8" t="n">
         <v>13429720</v>
-      </c>
-      <c r="G8" t="n">
-        <v>13207089</v>
       </c>
       <c r="H8" t="n">
         <v>13597066</v>
@@ -628,10 +628,10 @@
         <v>16</v>
       </c>
       <c r="B9" t="n">
+        <v>1325594</v>
+      </c>
+      <c r="C9" t="n">
         <v>1183205</v>
-      </c>
-      <c r="C9" t="n">
-        <v>1325594</v>
       </c>
       <c r="D9" t="n">
         <v>1119342</v>
@@ -640,10 +640,10 @@
         <v>1135888</v>
       </c>
       <c r="F9" t="n">
+        <v>1397493</v>
+      </c>
+      <c r="G9" t="n">
         <v>1283176</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1397493</v>
       </c>
       <c r="H9" t="n">
         <v>1129050</v>

</xml_diff>